<commit_message>
Rename "period" to "lecture" throughout
User-facing: grid labels P1..P7 become L1..L7 (UI, PDF, Excel), the Excel
"Period" column becomes "Lecture", and messages say "lecture".
Data model and formats: periods_per_day -> lectures_per_day,
max_periods_per_day -> max_lectures_per_day, Slot.period -> Slot.lecture
(JSON API, Excel template keys and TypeScript types). This is a breaking
change for data written before this commit; the project is unreleased.

The template workbook is regenerated.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/institution-template.xlsx
+++ b/docs/institution-template.xlsx
@@ -433,7 +433,7 @@
   <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="31" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -476,7 +476,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>periods_per_day</t>
+          <t>lectures_per_day</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -699,7 +699,7 @@
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -721,7 +721,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>max_periods_per_day</t>
+          <t>max_lectures_per_day</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Add named home rooms for classes
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/institution-template.xlsx
+++ b/docs/institution-template.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Batches" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Courses" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Offerings" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Pins" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -430,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -498,51 +499,91 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>weight_repeat_course_day</t>
+          <t>early_lectures</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>weight_batch_gaps</t>
+          <t>late_lectures</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>weight_faculty_gaps</t>
+          <t>weight_repeat_course_day</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>weight_peak_day_load</t>
+          <t>weight_batch_gaps</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>weight_faculty_gaps</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>weight_peak_day_load</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>weight_avoid_slot</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B12" t="n">
         <v>6</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>weight_room_changes</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>weight_odd_hours</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1037,7 +1078,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1048,6 +1089,8 @@
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1091,6 +1134,16 @@
           <t>group_of</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>clock</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>home_room</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1125,6 +1178,8 @@
         <v>60</v>
       </c>
       <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1159,6 +1214,8 @@
         <v>55</v>
       </c>
       <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1193,6 +1250,8 @@
         <v>25</v>
       </c>
       <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1227,6 +1286,8 @@
         <v>60</v>
       </c>
       <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1261,6 +1322,8 @@
         <v>30</v>
       </c>
       <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1299,6 +1362,8 @@
           <t>CS-UG1</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1337,6 +1402,8 @@
           <t>CS-UG1</t>
         </is>
       </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1375,6 +1442,8 @@
           <t>CS-UG3</t>
         </is>
       </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1413,6 +1482,8 @@
           <t>CS-UG3</t>
         </is>
       </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -2951,4 +3022,52 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>offering_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>session</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>lecture</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>room</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add a goal for spreading a course's sessions over non-consecutive days
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/institution-template.xlsx
+++ b/docs/institution-template.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -583,6 +583,16 @@
         </is>
       </c>
       <c r="B14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>weight_day_spacing</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>